<commit_message>
Đồng bộ hai website theo app bản 375 (thêm Học tập và làm theo Bác — QĐ 2995, Tuần 9–10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/Dao duc - Lop 1.xlsx
+++ b/assets/docs/lop1/Dao duc - Lop 1.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: Tự chăm sóc</t>
+          <t>Chủ đề 1: Tự chăm sóc bản thân</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -570,7 +570,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: Tự chăm sóc</t>
+          <t>Chủ đề 1: Tự chăm sóc bản thân</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: Tự chăm sóc</t>
+          <t>Chủ đề 1: Tự chăm sóc bản thân</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
@@ -640,7 +640,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CĐ 1: Tự chăm sóc</t>
+          <t>Chủ đề 1: Tự chăm sóc bản thân</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CĐ 2: Yêu thương</t>
+          <t>Chủ đề 2: Yêu thương gia đình</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CĐ 2: Yêu thương</t>
+          <t>Chủ đề 2: Yêu thương gia đình</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>

</xml_diff>